<commit_message>
fix: secure children data download to admin only and fix excel export corruption
</commit_message>
<xml_diff>
--- a/server/uploads/children_records.xlsx
+++ b/server/uploads/children_records.xlsx
@@ -397,24 +397,63 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1"/>
+  <dimension ref="A1:L1"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="22.83203125" customWidth="1"/>
-    <col min="4" max="4" width="6.83203125" customWidth="1"/>
+    <col min="3" max="3" width="24.83203125" customWidth="1"/>
+    <col min="4" max="4" width="8.83203125" customWidth="1"/>
     <col min="5" max="5" width="10.83203125" customWidth="1"/>
-    <col min="6" max="6" width="15.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="16.83203125" customWidth="1"/>
-    <col min="10" max="10" width="30.83203125" customWidth="1"/>
-    <col min="11" max="11" width="25.83203125" customWidth="1"/>
-    <col min="12" max="12" width="25.83203125" customWidth="1"/>
+    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="25.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="32.83203125" customWidth="1"/>
+    <col min="11" max="11" width="28.83203125" customWidth="1"/>
+    <col min="12" max="12" width="28.83203125" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>S.No</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Serial ID</v>
+      </c>
+      <c r="C1" t="str">
+        <v>Full Name</v>
+      </c>
+      <c r="D1" t="str">
+        <v>Age</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Gender</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Class / Grade</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Admission Date</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Guardian / Parent Name</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Guardian Phone</v>
+      </c>
+      <c r="J1" t="str">
+        <v>Address / Native Place</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Medical &amp; Health Notes</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Hobbies &amp; Talents</v>
+      </c>
+    </row>
+  </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>